<commit_message>
Refresh September S1 and E10 in isolation and realize BUIDL cash variances
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-09/grove_settlement_september_2026.xlsx
+++ b/settlements/grove/2026-09/grove_settlement_september_2026.xlsx
@@ -7,13 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Close status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Venues" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sky Revenue" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sky Direct" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Debt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Off-protocol holdings" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Off-protocol holdings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -78,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -92,12 +91,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -465,144 +458,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="115" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>September 2026 close</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>Official reference-rate coverage complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>calculation</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>Independent full monthly pipeline, compared field-by-field with September 30 API result</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>calculation_code_version</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>c32f25a7ef410eaaf9212b8f546f652c715dc7ac</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>daily_revision</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>11c4df339ebe710cccc6890a674ec4bdb35df3248ec76944050fe24fef4363cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>monthly_result_sha256</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>b65cbc633943ce542f7817074640dc81c3a138e0ad9301767dd12f7bc618afc6</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>daily_result_sha256</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>b65cbc633943ce542f7817074640dc81c3a138e0ad9301767dd12f7bc618afc6</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>all result fields match</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>distribution_rewards_workbook_sha256</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>17eee2ca39bd63e68e6d87097ede0007d8741e41cb9a7fceb017da713103b02e</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>distribution_rewards_code</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>1e9ecb2 (merged settle-dr-dune PR #27; finalized September snapshot)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>reference_rate_status</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>official coverage complete</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -670,6 +525,7 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr"/>
       <c r="B8" s="4" t="n">
         <v>4903217.156937339</v>
       </c>
@@ -693,7 +549,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>3754292.984290455</v>
+        <v>3754809.063890275</v>
       </c>
     </row>
     <row r="12">
@@ -703,12 +559,13 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>2507467.934719144</v>
+        <v>2175801.855496144</v>
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr"/>
       <c r="B13" s="4" t="n">
-        <v>6261760.919009599</v>
+        <v>5930610.919386419</v>
       </c>
     </row>
     <row r="15">
@@ -730,7 +587,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>3754292.984290455</v>
+        <v>3754809.063890275</v>
       </c>
     </row>
     <row r="17">
@@ -740,10 +597,11 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>-2825885.752437733</v>
+        <v>-2825369.672837913</v>
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr"/>
       <c r="B18" s="4" t="n">
         <v>6580178.736728188</v>
       </c>
@@ -777,12 +635,13 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>-3754292.984290455</v>
+        <v>-3754809.063890275</v>
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr"/>
       <c r="B23" s="4" t="n">
-        <v>1041914.638349169</v>
+        <v>1041398.558749349</v>
       </c>
     </row>
     <row r="25">
@@ -817,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-01T15:36:05+00:00</t>
+          <t>2026-10-01T16:21:52+00:00</t>
         </is>
       </c>
     </row>
@@ -838,7 +697,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1037,12 +896,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E42</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
+          <t>Galaxy Warehouse (off-chain facility — cash distribution to Grove Eth ALM)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1052,113 +911,113 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>643254421.77</v>
+        <v>0</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>119322905.35</v>
+        <v>0</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-523931516.42</v>
+        <v>0</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>1065483.58</v>
+        <v>1658948.54</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0</v>
+        <v>1658948.54</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>1065483.58</v>
+        <v>0</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>335756055.1033334</v>
+        <v>304000001</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>0</v>
+        <v>957291.5235085657</v>
       </c>
       <c r="O3" s="5" t="n">
-        <v>1065483.58</v>
+        <v>957291.5235085657</v>
       </c>
       <c r="P3" s="5" t="n">
-        <v>0</v>
+        <v>701657.0164914343</v>
       </c>
       <c r="Q3" s="5" t="n">
-        <v>335756055.1033334</v>
+        <v>0</v>
       </c>
       <c r="R3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>SDE (fixed)</t>
+          <t>(off-chain notional)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E42</t>
+          <t>E20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Galaxy Warehouse (off-chain facility — cash distribution to Grove Eth ALM)</t>
+          <t>Janus Henderson Anemoy AAA CLO (JAAA-avalanche)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>avalanche_c</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0</v>
+        <v>261874260.001064</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0</v>
+        <v>262568675.088451</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0</v>
+        <v>694415.0873870148</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>1658948.54</v>
+        <v>694415.0873870148</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>1658948.54</v>
+        <v>694415.0873870148</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>304000001</v>
+        <v>261874260.001064</v>
       </c>
       <c r="M4" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>957159.948608762</v>
+        <v>824638.1858534823</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>957159.948608762</v>
+        <v>824638.1858534823</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>701788.591391238</v>
+        <v>-130223.0984664676</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1166,26 +1025,22 @@
       <c r="R4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>(off-chain notional)</t>
-        </is>
-      </c>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E20</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Janus Henderson Anemoy AAA CLO (JAAA-avalanche)</t>
+          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1194,46 +1049,51 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>261874260.001064</v>
+        <v>643254421.77</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>262568675.088451</v>
+        <v>119263243.897325</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>694415.0873870148</v>
+        <v>-523991177.872675</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>694415.0873870148</v>
+        <v>733817.500777</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>694415.0873870148</v>
+        <v>0</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>0</v>
+        <v>733817.500777</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>261874260.001064</v>
+        <v>335908171.77</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>824524.8434870105</v>
+        <v>0</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>824524.8434870105</v>
+        <v>733817.500777</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>-130109.7560999957</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>0</v>
+        <v>335908171.77</v>
       </c>
       <c r="R5" s="5" t="n">
         <v>0</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>SDE (fixed)</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1285,13 +1145,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>635116.405302843</v>
+        <v>635203.7108545565</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>635116.405302843</v>
+        <v>635203.7108545565</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>75849.9442576921</v>
+        <v>75762.63870597855</v>
       </c>
       <c r="Q6" s="5" t="n">
         <v>0</v>
@@ -1299,6 +1159,7 @@
       <c r="R6" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1349,13 +1210,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>411625.9330412184</v>
+        <v>411682.5167302614</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>411625.9330412184</v>
+        <v>411682.5167302614</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>-64954.44033672687</v>
+        <v>-65011.02402576988</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1363,6 +1224,7 @@
       <c r="R7" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1413,13 +1275,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>324521.2817243162</v>
+        <v>324565.8916718899</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>324521.2817243162</v>
+        <v>324565.8916718899</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>11053.71827568376</v>
+        <v>11009.1083281101</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1427,6 +1289,7 @@
       <c r="R8" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1477,13 +1340,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>255083.6543830937</v>
+        <v>255118.7191664831</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>255083.6543830937</v>
+        <v>255118.7191664831</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>26530.78653668918</v>
+        <v>26495.72175329974</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1491,6 +1354,7 @@
       <c r="R9" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1541,13 +1405,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>122172.7803888801</v>
+        <v>122189.5747306845</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>122172.7803888801</v>
+        <v>122189.5747306845</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>-122172.7803888801</v>
+        <v>-122189.5747306845</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1555,6 +1419,7 @@
       <c r="R10" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1605,13 +1470,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>78713.81130429354</v>
+        <v>78724.63160851813</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>78713.81130429354</v>
+        <v>78724.63160851813</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-65896.44655329354</v>
+        <v>-65907.26685751813</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1674,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>65186.97496370061</v>
+        <v>65195.93581680757</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>65186.97496370061</v>
+        <v>65195.93581680757</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-169625.2528326332</v>
+        <v>-169634.2136857402</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1688,6 +1553,7 @@
       <c r="R12" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1738,13 +1604,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>56383.75714114093</v>
+        <v>56391.50786995819</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>56383.75714114093</v>
+        <v>56391.50786995819</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>115783.5828588591</v>
+        <v>115775.8321300418</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1752,6 +1618,7 @@
       <c r="R13" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1802,13 +1669,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>21130.19404277929</v>
+        <v>21133.09868078473</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>21130.19404277929</v>
+        <v>21133.09868078473</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>1168.090225019724</v>
+        <v>1165.185587014287</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1816,6 +1683,7 @@
       <c r="R14" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1866,13 +1734,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>2230.224653621651</v>
+        <v>2230.531228908013</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>2230.224653621651</v>
+        <v>2230.531228908013</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>-2230.224653621651</v>
+        <v>-2230.531228908013</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1880,6 +1748,7 @@
       <c r="R15" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1930,13 +1799,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>411.4712407511063</v>
+        <v>411.5278031755502</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>411.4712407511063</v>
+        <v>411.5278031755502</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>-411.4712407511063</v>
+        <v>-411.5278031755502</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1944,6 +1813,7 @@
       <c r="R16" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1994,13 +1864,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>31.7027080364387</v>
+        <v>31.70706601301248</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>31.7027080364387</v>
+        <v>31.70706601301248</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-31.7027080364387</v>
+        <v>-31.70706601301248</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -2008,6 +1878,7 @@
       <c r="R17" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2058,13 +1929,13 @@
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.001165700753062453</v>
+        <v>0.001165860994785906</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>0.001165700753062453</v>
+        <v>0.001165860994785906</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>-0.0004511203258199923</v>
+        <v>-0.0004512805675434453</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -2072,6 +1943,7 @@
       <c r="R18" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2122,13 +1994,13 @@
         <v>1</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>8.937090443336482e-05</v>
+        <v>8.938318970273206e-05</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>8.937090443336482e-05</v>
+        <v>8.938318970273206e-05</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>9.33488075948298e-05</v>
+        <v>9.333652232546256e-05</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>0</v>
@@ -2136,6 +2008,7 @@
       <c r="R19" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2186,13 +2059,13 @@
         <v>1</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>4.49325459406089e-05</v>
+        <v>4.493872254174923e-05</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>4.49325459406089e-05</v>
+        <v>4.493872254174923e-05</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>-2.42997255811159e-05</v>
+        <v>-2.430590218225623e-05</v>
       </c>
       <c r="Q20" s="5" t="n">
         <v>0</v>
@@ -2200,6 +2073,7 @@
       <c r="R20" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2250,13 +2124,13 @@
         <v>1</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>3.148552452171742e-09</v>
+        <v>3.148985264340725e-09</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>3.148552452171742e-09</v>
+        <v>3.148985264340725e-09</v>
       </c>
       <c r="P21" s="5" t="n">
-        <v>-3.148552452171742e-09</v>
+        <v>-3.148985264340725e-09</v>
       </c>
       <c r="Q21" s="5" t="n">
         <v>0</v>
@@ -2264,6 +2138,7 @@
       <c r="R21" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2328,6 +2203,7 @@
       <c r="R22" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2392,6 +2268,7 @@
       <c r="R23" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2456,6 +2333,7 @@
       <c r="R24" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2520,6 +2398,7 @@
       <c r="R25" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2584,6 +2463,7 @@
       <c r="R26" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2648,6 +2528,7 @@
       <c r="R27" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2712,6 +2593,7 @@
       <c r="R28" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2845,6 +2727,7 @@
       <c r="R30" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2909,6 +2792,7 @@
       <c r="R31" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2973,6 +2857,7 @@
       <c r="R32" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3037,6 +2922,7 @@
       <c r="R33" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3101,6 +2987,7 @@
       <c r="R34" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="S34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3113,6 +3000,8 @@
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" s="5" t="n">
         <v>0</v>
       </c>
@@ -3166,7 +3055,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3212,7 +3101,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1231235574.391315</v>
+        <v>1231403801.339027</v>
       </c>
     </row>
     <row r="6">
@@ -3232,7 +3121,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>231235574.3913149</v>
+        <v>231403801.3390272</v>
       </c>
     </row>
     <row r="8">
@@ -3242,7 +3131,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.03737049927466624</v>
+        <v>0.03737049297570649</v>
       </c>
     </row>
     <row r="9">
@@ -3272,7 +3161,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>0.03709869358790142</v>
+        <v>0.03709872442139246</v>
       </c>
     </row>
     <row r="12">
@@ -3282,7 +3171,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>-2.718056867648138</v>
+        <v>-2.717685543140242</v>
       </c>
     </row>
     <row r="13">
@@ -3302,7 +3191,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>3781799.025183608</v>
+        <v>3782315.104783428</v>
       </c>
     </row>
     <row r="16">
@@ -3312,7 +3201,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>3754292.984290455</v>
+        <v>3754809.063890275</v>
       </c>
     </row>
     <row r="17">
@@ -3362,10 +3251,10 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>231235574.3913149</v>
+        <v>231403801.3390272</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>710483.9572981695</v>
+        <v>711000.0368979895</v>
       </c>
     </row>
     <row r="23">
@@ -3387,7 +3276,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>3754292.984290455</v>
+        <v>3754809.063890275</v>
       </c>
     </row>
     <row r="25">
@@ -3397,7 +3286,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>2507467.934719144</v>
+        <v>2175801.855496144</v>
       </c>
     </row>
     <row r="26">
@@ -3407,7 +3296,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>6261760.919009599</v>
+        <v>5930610.919386419</v>
       </c>
     </row>
     <row r="28">
@@ -3434,7 +3323,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>3754292.984290455</v>
+        <v>3754809.063890275</v>
       </c>
     </row>
     <row r="32">
@@ -3444,7 +3333,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>-2825885.752437733</v>
+        <v>-2825369.672837913</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -3558,7 +3447,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3649,6 +3538,7 @@
           <t>fixed</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>2025-10-30</t>
@@ -3675,10 +3565,10 @@
         </is>
       </c>
       <c r="I4" s="5" t="n">
-        <v>1065483.58</v>
+        <v>733817.500777</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>1065483.58</v>
+        <v>733817.500777</v>
       </c>
     </row>
     <row r="5">
@@ -3692,6 +3582,7 @@
           <t>fixed</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>2025-10-30</t>
@@ -3775,7 +3666,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3913,7 +3804,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1451451703.157209</v>
+        <v>1451142543.444814</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0</v>
@@ -3925,7 +3816,7 @@
         <v>12499999.49993904</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>1162714094.46428</v>
+        <v>1163023254.176675</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>0.03519999850777533</v>
@@ -3943,7 +3834,7 @@
         <v>0.03661485249996968</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>116650.5164126346</v>
+        <v>116681.5548259428</v>
       </c>
       <c r="P6" s="3" t="n">
         <v>263625.481741702</v>
@@ -3965,7 +3856,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1426577413.99278</v>
+        <v>1426268224.416485</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0</v>
@@ -3977,7 +3868,7 @@
         <v>12499999.49993904</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>1164710678.150574</v>
+        <v>1165019867.726869</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>0.03519999850777533</v>
@@ -3995,7 +3886,7 @@
         <v>0.03654818583330301</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>116668.3171223034</v>
+        <v>116699.3585338292</v>
       </c>
       <c r="P7" s="3" t="n">
         <v>261146.0021238221</v>
@@ -4017,7 +3908,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>1401714968.754915</v>
+        <v>1401418249.31338</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>0</v>
@@ -4029,7 +3920,7 @@
         <v>12499997.4905512</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>1159517150.935699</v>
+        <v>1159813870.377234</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4047,7 +3938,7 @@
         <v>0.03687310577117104</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>117375.6949561137</v>
+        <v>117406.1142408696</v>
       </c>
       <c r="P8" s="3" t="n">
         <v>262359.1430970955</v>
@@ -4069,7 +3960,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>1351879932.737562</v>
+        <v>1351595684.548662</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>0</v>
@@ -4081,7 +3972,7 @@
         <v>12499999.4999392</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>1204346251.38071</v>
+        <v>1204630499.56961</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4099,7 +3990,7 @@
         <v>0.03680643910450437</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>121788.8666486194</v>
+        <v>121818.0073970474</v>
       </c>
       <c r="P9" s="3" t="n">
         <v>261663.2930063853</v>
@@ -4121,7 +4012,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1351879932.737562</v>
+        <v>1351595684.548662</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0</v>
@@ -4133,7 +4024,7 @@
         <v>12499999.4999392</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>1204346251.38071</v>
+        <v>1204630499.56961</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4151,7 +4042,7 @@
         <v>0.03680643910450437</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>121788.8666486194</v>
+        <v>121818.0073970474</v>
       </c>
       <c r="P10" s="3" t="n">
         <v>261663.2930063853</v>
@@ -4173,7 +4064,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>1351879932.737562</v>
+        <v>1351595684.548662</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0</v>
@@ -4185,7 +4076,7 @@
         <v>12499999.4999392</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>1204346251.38071</v>
+        <v>1204630499.56961</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4203,7 +4094,7 @@
         <v>0.03680643910450437</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>121788.8666486194</v>
+        <v>121818.0073970474</v>
       </c>
       <c r="P11" s="3" t="n">
         <v>261663.2930063853</v>
@@ -4225,7 +4116,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>1351879932.737562</v>
+        <v>1351595684.548662</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
@@ -4237,7 +4128,7 @@
         <v>12499999.4999392</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>1204346251.38071</v>
+        <v>1204630499.56961</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4255,7 +4146,7 @@
         <v>0.03680643910450437</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>121788.8666486194</v>
+        <v>121818.0073970474</v>
       </c>
       <c r="P12" s="3" t="n">
         <v>261663.2930063853</v>
@@ -4277,7 +4168,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1327389909.500666</v>
+        <v>1327105546.471406</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0</v>
@@ -4289,7 +4180,7 @@
         <v>12499999.4999392</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>1178401441.817879</v>
+        <v>1178685804.84714</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4307,7 +4198,7 @@
         <v>0.03673977243783771</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>118946.3906805731</v>
+        <v>118975.543202283</v>
       </c>
       <c r="P13" s="3" t="n">
         <v>256310.1322424029</v>
@@ -4329,7 +4220,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>1277499086.469848</v>
+        <v>1277227195.919933</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>0</v>
@@ -4341,7 +4232,7 @@
         <v>12499999.4999392</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>1170394488.290329</v>
+        <v>1170666378.840244</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4359,7 +4250,7 @@
         <v>0.03673977243783771</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>118125.528393554</v>
+        <v>118153.4022531754</v>
       </c>
       <c r="P14" s="3" t="n">
         <v>250374.5287553221</v>
@@ -4381,7 +4272,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>1252604939.361961</v>
+        <v>1252345522.555306</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>0</v>
@@ -4393,7 +4284,7 @@
         <v>12499999.4999392</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>1160130042.603527</v>
+        <v>1160389459.410182</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4411,7 +4302,7 @@
         <v>0.03660643910450437</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>116707.934192088</v>
+        <v>116734.529260046</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>246404.8195130909</v>
@@ -4433,7 +4324,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1202672621.804375</v>
+        <v>1202425680.058425</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>0</v>
@@ -4445,7 +4336,7 @@
         <v>12349466.27698199</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>1188971884.251625</v>
+        <v>1189218825.997575</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4463,7 +4354,7 @@
         <v>0.03660643910450437</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>119664.7616565709</v>
+        <v>119690.0777978028</v>
       </c>
       <c r="P16" s="3" t="n">
         <v>244227.2193465533</v>
@@ -4485,7 +4376,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>1202672621.804375</v>
+        <v>1202425680.058425</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>0</v>
@@ -4497,7 +4388,7 @@
         <v>12349466.27698199</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>1236471884.251625</v>
+        <v>1236718825.997575</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4515,7 +4406,7 @@
         <v>0.03660643910450437</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>124534.3988412062</v>
+        <v>124559.7149824381</v>
       </c>
       <c r="P17" s="3" t="n">
         <v>249096.8565311886</v>
@@ -4537,7 +4428,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>1202672621.804375</v>
+        <v>1202425680.058425</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>0</v>
@@ -4549,7 +4440,7 @@
         <v>12349466.27698199</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>1243605525.600235</v>
+        <v>1243852467.346184</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4567,7 +4458,7 @@
         <v>0.03660643910450437</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>125265.7303185334</v>
+        <v>125291.0464597653</v>
       </c>
       <c r="P18" s="3" t="n">
         <v>249828.1880085158</v>
@@ -4589,7 +4480,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>1152947197.094734</v>
+        <v>1152712684.14362</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>0</v>
@@ -4601,7 +4492,7 @@
         <v>27349410.47621031</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>1223779320.334566</v>
+        <v>1224013833.285681</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4619,7 +4510,7 @@
         <v>0.03660643910450437</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>123233.1739734405</v>
+        <v>123257.2159310622</v>
       </c>
       <c r="P19" s="3" t="n">
         <v>244235.6213234686</v>
@@ -4641,7 +4532,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>1103045374.710737</v>
+        <v>1102823339.212842</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0</v>
@@ -4653,7 +4544,7 @@
         <v>27349410.47621031</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>1224094368.44795</v>
+        <v>1224316403.945845</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4671,7 +4562,7 @@
         <v>0.03673977243783771</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>123630.7690930489</v>
+        <v>123653.531878667</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>239517.3476038732</v>
@@ -4693,7 +4584,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>828150477.9916395</v>
+        <v>828053420.9860544</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0</v>
@@ -4705,7 +4596,7 @@
         <v>42349410.4742758</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>1425840215.624381</v>
+        <v>1425937272.629966</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4723,7 +4614,7 @@
         <v>0.03660643910450437</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>143948.1897474189</v>
+        <v>143958.1399032806</v>
       </c>
       <c r="P21" s="3" t="n">
         <v>233190.6871388816</v>
@@ -4745,7 +4636,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>478207338.4712687</v>
+        <v>478135262.4845636</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0</v>
@@ -4757,7 +4648,7 @@
         <v>49999999.50293472</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>1230257992.339858</v>
+        <v>1230330068.326563</v>
       </c>
       <c r="J22" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4775,7 +4666,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>126124.4224461663</v>
+        <v>126131.811581008</v>
       </c>
       <c r="P22" s="3" t="n">
         <v>180275.5402187219</v>
@@ -4797,7 +4688,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>478261841.6359231</v>
+        <v>478189758.3260831</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>0</v>
@@ -4809,7 +4700,7 @@
         <v>49999999.50293472</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>1230410802.094075</v>
+        <v>1230482885.403915</v>
       </c>
       <c r="J23" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4827,7 +4718,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>126140.0883000887</v>
+        <v>126147.4781856885</v>
       </c>
       <c r="P23" s="3" t="n">
         <v>180296.7936650081</v>
@@ -4849,7 +4740,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>478261841.6359231</v>
+        <v>478189758.3260831</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>0</v>
@@ -4861,7 +4752,7 @@
         <v>49999999.50293472</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>1230410802.094075</v>
+        <v>1230482885.403915</v>
       </c>
       <c r="J24" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4879,7 +4770,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>126140.0883000887</v>
+        <v>126147.4781856885</v>
       </c>
       <c r="P24" s="3" t="n">
         <v>180296.7936650081</v>
@@ -4901,7 +4792,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>478261841.6359231</v>
+        <v>478189758.3260831</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>0</v>
@@ -4913,7 +4804,7 @@
         <v>49999999.50293472</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>1230410802.094075</v>
+        <v>1230482885.403915</v>
       </c>
       <c r="J25" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4931,7 +4822,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>126140.0883000887</v>
+        <v>126147.4781856885</v>
       </c>
       <c r="P25" s="3" t="n">
         <v>180296.7936650081</v>
@@ -4953,7 +4844,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>453400872.6759484</v>
+        <v>453341267.3985784</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>0</v>
@@ -4965,7 +4856,7 @@
         <v>49999999.50293472</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>1263329378.267849</v>
+        <v>1263388983.545219</v>
       </c>
       <c r="J26" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -4983,7 +4874,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>129514.8571969531</v>
+        <v>129520.9678511653</v>
       </c>
       <c r="P26" s="3" t="n">
         <v>181122.8489009555</v>
@@ -5005,7 +4896,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>428443877.0686115</v>
+        <v>428384264.4666215</v>
       </c>
       <c r="F27" s="5" t="n">
         <v>0</v>
@@ -5017,7 +4908,7 @@
         <v>49999999.49992944</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>1253846911.286531</v>
+        <v>1253906523.888521</v>
       </c>
       <c r="J27" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5035,7 +4926,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>128542.7272219151</v>
+        <v>128548.8386270378</v>
       </c>
       <c r="P27" s="3" t="n">
         <v>177592.1607397933</v>
@@ -5057,7 +4948,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>428488742.6539316</v>
+        <v>428429123.9705616</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0</v>
@@ -5069,7 +4960,7 @@
         <v>49999999.49992944</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>1263779186.409572</v>
+        <v>1263838805.092942</v>
       </c>
       <c r="J28" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5087,7 +4978,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>129560.9709328033</v>
+        <v>129567.082961381</v>
       </c>
       <c r="P28" s="3" t="n">
         <v>178615.004011157</v>
@@ -5109,7 +5000,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>428520425.1043783</v>
+        <v>428460800.3391283</v>
       </c>
       <c r="F29" s="5" t="n">
         <v>0</v>
@@ -5121,7 +5012,7 @@
         <v>49999999.49992944</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>1268387920.776347</v>
+        <v>1268447545.541597</v>
       </c>
       <c r="J29" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5139,7 +5030,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>130033.4522853624</v>
+        <v>130039.5649374463</v>
       </c>
       <c r="P29" s="3" t="n">
         <v>179090.7334066381</v>
@@ -5161,7 +5052,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>428555179.9442062</v>
+        <v>428495549.0795212</v>
       </c>
       <c r="F30" s="5" t="n">
         <v>0</v>
@@ -5173,7 +5064,7 @@
         <v>64999999.49992924</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>1261885882.043658</v>
+        <v>1261945512.908344</v>
       </c>
       <c r="J30" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5191,7 +5082,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>129366.87187297</v>
+        <v>129372.9851503599</v>
       </c>
       <c r="P30" s="3" t="n">
         <v>179965.496178033</v>
@@ -5213,7 +5104,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>428555179.9442062</v>
+        <v>428495549.0795212</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>0</v>
@@ -5225,7 +5116,7 @@
         <v>79996199.75835411</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>1261885882.043659</v>
+        <v>1261945512.908344</v>
       </c>
       <c r="J31" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5243,7 +5134,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>129366.87187297</v>
+        <v>129372.9851503599</v>
       </c>
       <c r="P31" s="3" t="n">
         <v>181502.8867971206</v>
@@ -5265,7 +5156,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>428555179.9442062</v>
+        <v>428495549.0795212</v>
       </c>
       <c r="F32" s="5" t="n">
         <v>0</v>
@@ -5277,7 +5168,7 @@
         <v>79996199.75835411</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>1263152362.795656</v>
+        <v>1263211993.660341</v>
       </c>
       <c r="J32" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5295,7 +5186,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>129496.7098048342</v>
+        <v>129502.8230822241</v>
       </c>
       <c r="P32" s="3" t="n">
         <v>181632.7247289848</v>
@@ -5317,7 +5208,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>428678718.9430575</v>
+        <v>428619069.7155825</v>
       </c>
       <c r="F33" s="5" t="n">
         <v>0</v>
@@ -5329,7 +5220,7 @@
         <v>79996199.75835411</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>1268735358.038735</v>
+        <v>1268795007.26621</v>
       </c>
       <c r="J33" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5347,7 +5238,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>130069.0710940414</v>
+        <v>130075.1862539603</v>
       </c>
       <c r="P33" s="3" t="n">
         <v>182217.7510729828</v>
@@ -5369,7 +5260,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>428722277.2711748</v>
+        <v>428662621.9223148</v>
       </c>
       <c r="F34" s="5" t="n">
         <v>0</v>
@@ -5381,7 +5272,7 @@
         <v>99999999.49992901</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>1269927335.970441</v>
+        <v>1269986991.319301</v>
       </c>
       <c r="J34" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5399,7 +5290,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>130191.271095294</v>
+        <v>130197.3868827692</v>
       </c>
       <c r="P34" s="3" t="n">
         <v>184395.1797123379</v>
@@ -5421,7 +5312,7 @@
         <v>0</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>428783732.5412791</v>
+        <v>428724071.0886041</v>
       </c>
       <c r="F35" s="5" t="n">
         <v>0</v>
@@ -5433,7 +5324,7 @@
         <v>99999999.49992901</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>1284630515.189406</v>
+        <v>1284690176.642081</v>
       </c>
       <c r="J35" s="6" t="n">
         <v>0.03600000425292382</v>
@@ -5451,7 +5342,7 @@
         <v>0.03741931731351311</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>131698.6215849156</v>
+        <v>131704.7379981459</v>
       </c>
       <c r="P35" s="3" t="n">
         <v>185908.8305149805</v>
@@ -5463,8 +5354,21 @@
           <t>Σ daily charges</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" s="10" t="n">
-        <v>3754292.984290455</v>
+        <v>3754809.063890275</v>
       </c>
       <c r="P37" s="10" t="n">
         <v>6580178.736728188</v>
@@ -5475,7 +5379,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5572,6 +5476,8 @@
           <t>monad</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" s="5" t="n">
         <v>0</v>
       </c>
@@ -5603,6 +5509,8 @@
           <t>ethereum</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" s="5" t="n">
         <v>0</v>
       </c>
@@ -5675,6 +5583,8 @@
           <t>monad</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" s="5" t="n">
         <v>0</v>
       </c>
@@ -5706,6 +5616,8 @@
           <t>monad</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" s="5" t="n">
         <v>0</v>
       </c>
@@ -5737,6 +5649,8 @@
           <t>monad</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" s="5" t="n">
         <v>152288.12728</v>
       </c>

</xml_diff>